<commit_message>
Add RC column design (axial-load P-M interaction)
- design/column.py: tied rectangular columns, symmetric two-face steel,
  ACI 318-19 strain-compatibility P-M interaction (phi 0.90/0.65 with
  linear transition), phi*Pn,max = 0.80 phi Po, tie spacing 25.7.2.1;
  NSCP 2015 equivalences noted per formula.
- design_members now routes near-vertical members (|dy| >= |dx| from
  optional node coordinates added by bridge/run.py) to column design;
  beam output keys unchanged, extended with type/axial/capacity/util/ok.
- workbook_layout: Outputs-Design gains type, Pu, phi*Pn, phi*Mn,
  utilization columns; demo workbook regenerated.
- sanity_check: hand-computable column cases (pure axial 0.80 phi Po,
  tension-controlled interaction point at c = 0.375 d, design passes and
  axial/moment over-capacity failures).
- README, docs/excel-bridge-architecture.md, examples/README, AGENTS.md
  updated; biaxial bending, slenderness, spirals documented as future work.
</commit_message>
<xml_diff>
--- a/examples/rc_matrix_solver_demo.xlsx
+++ b/examples/rc_matrix_solver_demo.xlsx
@@ -57,9 +57,14 @@
     <definedName name="OUT_MF_M_I">'Outputs-MemberForces'!$D$2:$D$1000</definedName>
     <definedName name="OUT_MF_M_J">'Outputs-MemberForces'!$E$2:$E$1000</definedName>
     <definedName name="OUT_DES_MEMBER_ID">'Outputs-Design'!$A$2:$A$1000</definedName>
-    <definedName name="OUT_DES_AS_REQ">'Outputs-Design'!$B$2:$B$1000</definedName>
-    <definedName name="OUT_DES_AS_PROV">'Outputs-Design'!$C$2:$C$1000</definedName>
-    <definedName name="OUT_DES_STIRRUP">'Outputs-Design'!$D$2:$D$1000</definedName>
+    <definedName name="OUT_DES_TYPE">'Outputs-Design'!$B$2:$B$1000</definedName>
+    <definedName name="OUT_DES_AS_REQ">'Outputs-Design'!$C$2:$C$1000</definedName>
+    <definedName name="OUT_DES_AS_PROV">'Outputs-Design'!$D$2:$D$1000</definedName>
+    <definedName name="OUT_DES_STIRRUP">'Outputs-Design'!$E$2:$E$1000</definedName>
+    <definedName name="OUT_DES_AXIAL_KN">'Outputs-Design'!$F$2:$F$1000</definedName>
+    <definedName name="OUT_DES_PHI_PN_KN">'Outputs-Design'!$G$2:$G$1000</definedName>
+    <definedName name="OUT_DES_PHI_MN_KNM">'Outputs-Design'!$H$2:$H$1000</definedName>
+    <definedName name="OUT_DES_UTIL">'Outputs-Design'!$I$2:$I$1000</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -4035,7 +4040,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1001"/>
+  <dimension ref="A1:I1001"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4046,17 +4051,42 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Design type</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>As required (mm^2)</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>As provided (mm^2)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Stirrup spacing (mm)</t>
+          <t>Stirrup/tie spacing (mm)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Axial Pu (kN)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Capacity phi*Pn (kN)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Capacity phi*Mn (kN*m)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Utilization</t>
         </is>
       </c>
     </row>
@@ -4064,28 +4094,62 @@
       <c r="A2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" t="n">
-        <v>912.2600115474009</v>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>COLUMN</t>
+        </is>
       </c>
       <c r="C2" t="n">
-        <v>1017.876019763093</v>
+        <v>1963.495408493621</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>1963.495408493621</v>
+      </c>
+      <c r="E2" t="n">
+        <v>390</v>
+      </c>
+      <c r="F2" t="n">
+        <v>53.38236501664918</v>
+      </c>
+      <c r="G2" t="n">
+        <v>2384.68717803949</v>
+      </c>
+      <c r="H2" t="n">
+        <v>129.0175627001236</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.8548773344622259</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
         <v>2</v>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>BEAM</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
         <v>439.9999999999999</v>
       </c>
-      <c r="C3" t="n">
+      <c r="D3" t="n">
         <v>490.8738521234052</v>
       </c>
-      <c r="D3" t="n">
+      <c r="E3" t="n">
         <v>220</v>
+      </c>
+      <c r="F3" t="n">
+        <v>1.818989403545856e-12</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>78.96326266081115</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.5028390236439734</v>
       </c>
     </row>
     <row r="4"/>

</xml_diff>